<commit_message>
Name the tournament and add T20 format to fixtures
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015MsuMnBjqU5knhALJ8GpAM
</commit_message>
<xml_diff>
--- a/cricket-whatsapp-helpdesk/tournament-fixtures-template.xlsx
+++ b/cricket-whatsapp-helpdesk/tournament-fixtures-template.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -424,6 +424,7 @@
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -462,6 +463,11 @@
           <t>Stage</t>
         </is>
       </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Format</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -497,6 +503,11 @@
           <t>League</t>
         </is>
       </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -532,6 +543,11 @@
           <t>League</t>
         </is>
       </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -567,6 +583,11 @@
           <t>League</t>
         </is>
       </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -602,6 +623,11 @@
           <t>League</t>
         </is>
       </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -637,6 +663,11 @@
           <t>League</t>
         </is>
       </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -672,6 +703,11 @@
           <t>League</t>
         </is>
       </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -707,6 +743,11 @@
           <t>League</t>
         </is>
       </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -742,6 +783,11 @@
           <t>League</t>
         </is>
       </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -777,6 +823,11 @@
           <t>League</t>
         </is>
       </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -812,6 +863,11 @@
           <t>League</t>
         </is>
       </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -847,6 +903,11 @@
           <t>League</t>
         </is>
       </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -882,6 +943,11 @@
           <t>League</t>
         </is>
       </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -917,6 +983,11 @@
           <t>Semi Final 1</t>
         </is>
       </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -952,6 +1023,11 @@
           <t>Semi Final 2</t>
         </is>
       </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -985,6 +1061,11 @@
       <c r="G16" t="inlineStr">
         <is>
           <t>Final</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>T20</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Name the tournament and add T20 format to fixtures (#2)
Claude-Session: https://claude.ai/code/session_015MsuMnBjqU5knhALJ8GpAM

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cricket-whatsapp-helpdesk/tournament-fixtures-template.xlsx
+++ b/cricket-whatsapp-helpdesk/tournament-fixtures-template.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G16"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -424,6 +424,7 @@
     <col width="22" customWidth="1" min="5" max="5"/>
     <col width="22" customWidth="1" min="6" max="6"/>
     <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -462,6 +463,11 @@
           <t>Stage</t>
         </is>
       </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Format</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -497,6 +503,11 @@
           <t>League</t>
         </is>
       </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -532,6 +543,11 @@
           <t>League</t>
         </is>
       </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -567,6 +583,11 @@
           <t>League</t>
         </is>
       </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -602,6 +623,11 @@
           <t>League</t>
         </is>
       </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -637,6 +663,11 @@
           <t>League</t>
         </is>
       </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -672,6 +703,11 @@
           <t>League</t>
         </is>
       </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -707,6 +743,11 @@
           <t>League</t>
         </is>
       </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -742,6 +783,11 @@
           <t>League</t>
         </is>
       </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -777,6 +823,11 @@
           <t>League</t>
         </is>
       </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -812,6 +863,11 @@
           <t>League</t>
         </is>
       </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -847,6 +903,11 @@
           <t>League</t>
         </is>
       </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -882,6 +943,11 @@
           <t>League</t>
         </is>
       </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -917,6 +983,11 @@
           <t>Semi Final 1</t>
         </is>
       </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -952,6 +1023,11 @@
           <t>Semi Final 2</t>
         </is>
       </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>T20</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -985,6 +1061,11 @@
       <c r="G16" t="inlineStr">
         <is>
           <t>Final</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>T20</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add results, points table, player stats and a 7-day tournament simulator
Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015MsuMnBjqU5knhALJ8GpAM
</commit_message>
<xml_diff>
--- a/cricket-whatsapp-helpdesk/tournament-fixtures-template.xlsx
+++ b/cricket-whatsapp-helpdesk/tournament-fixtures-template.xlsx
@@ -9,6 +9,8 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fixtures" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Squads" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Results" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Player Stats" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -414,17 +416,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -450,20 +453,25 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>Team A</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Team B</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Stage</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Format</t>
         </is>
@@ -475,7 +483,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>01 Nov 2026</t>
+          <t>17 Oct 2026</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -490,20 +498,25 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
           <t>Royal Strikers</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>Thunder Kings</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>League</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>T20</t>
         </is>
@@ -515,12 +528,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>01 Nov 2026</t>
+          <t>17 Oct 2026</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>01:30 PM</t>
+          <t>08:00 AM</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -530,7 +543,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Royal Strikers</t>
+          <t>A</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -540,10 +553,15 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
+          <t>Blue Warriors</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
           <t>League</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>T20</t>
         </is>
@@ -555,35 +573,40 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>02 Nov 2026</t>
+          <t>17 Oct 2026</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>01:30 PM</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>City Sports Complex</t>
+          <t>Academy Ground A</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Royal Strikers</t>
+          <t>B</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Blue Warriors</t>
+          <t>Eagle Eleven</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
+          <t>Lion Hearts</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
           <t>League</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>T20</t>
         </is>
@@ -595,12 +618,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>02 Nov 2026</t>
+          <t>18 Oct 2026</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>01:30 PM</t>
+          <t>08:00 AM</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -610,20 +633,25 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Royal Strikers</t>
+          <t>B</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Eagle Eleven</t>
+          <t>Storm Riders</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
+          <t>Golden Titans</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
           <t>League</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>T20</t>
         </is>
@@ -635,7 +663,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>03 Nov 2026</t>
+          <t>18 Oct 2026</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -650,20 +678,25 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
           <t>Royal Strikers</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Lion Hearts</t>
-        </is>
-      </c>
       <c r="G6" t="inlineStr">
         <is>
+          <t>Super Smashers</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
           <t>League</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>T20</t>
         </is>
@@ -675,7 +708,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>03 Nov 2026</t>
+          <t>18 Oct 2026</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -685,25 +718,30 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>City Sports Complex</t>
+          <t>Academy Ground A</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Royal Strikers</t>
+          <t>A</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Storm Riders</t>
+          <t>Thunder Kings</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
+          <t>Blue Warriors</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
           <t>League</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>T20</t>
         </is>
@@ -715,7 +753,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>04 Nov 2026</t>
+          <t>19 Oct 2026</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -730,20 +768,25 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Royal Strikers</t>
+          <t>B</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Golden Titans</t>
+          <t>Eagle Eleven</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
+          <t>Storm Riders</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
           <t>League</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>T20</t>
         </is>
@@ -755,12 +798,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>04 Nov 2026</t>
+          <t>19 Oct 2026</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>01:30 PM</t>
+          <t>08:00 AM</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -770,20 +813,25 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Thunder Kings</t>
+          <t>B</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Super Smashers</t>
+          <t>Lion Hearts</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
+          <t>Golden Titans</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
           <t>League</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>T20</t>
         </is>
@@ -795,35 +843,40 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>05 Nov 2026</t>
+          <t>19 Oct 2026</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>01:30 PM</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>City Sports Complex</t>
+          <t>Academy Ground A</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Thunder Kings</t>
+          <t>A</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
+          <t>Royal Strikers</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
           <t>Blue Warriors</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>League</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="I10" t="inlineStr">
         <is>
           <t>T20</t>
         </is>
@@ -835,12 +888,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>05 Nov 2026</t>
+          <t>20 Oct 2026</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>01:30 PM</t>
+          <t>08:00 AM</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -850,20 +903,25 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
           <t>Thunder Kings</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>Eagle Eleven</t>
-        </is>
-      </c>
       <c r="G11" t="inlineStr">
         <is>
+          <t>Super Smashers</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
           <t>League</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="I11" t="inlineStr">
         <is>
           <t>T20</t>
         </is>
@@ -875,7 +933,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>06 Nov 2026</t>
+          <t>20 Oct 2026</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -890,20 +948,25 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Thunder Kings</t>
+          <t>B</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Lion Hearts</t>
+          <t>Eagle Eleven</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
+          <t>Golden Titans</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
           <t>League</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>T20</t>
         </is>
@@ -915,7 +978,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>06 Nov 2026</t>
+          <t>20 Oct 2026</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -925,25 +988,30 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>City Sports Complex</t>
+          <t>Academy Ground A</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Thunder Kings</t>
+          <t>B</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
+          <t>Lion Hearts</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
           <t>Storm Riders</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="H13" t="inlineStr">
         <is>
           <t>League</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="I13" t="inlineStr">
         <is>
           <t>T20</t>
         </is>
@@ -955,7 +1023,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>07 Nov 2026</t>
+          <t>22 Oct 2026</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -968,22 +1036,23 @@
           <t>City Sports Complex</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
+      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Group A Winner</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
+          <t>Group B Runner-up</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
           <t>Semi Final 1</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="I14" t="inlineStr">
         <is>
           <t>T20</t>
         </is>
@@ -995,7 +1064,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>07 Nov 2026</t>
+          <t>22 Oct 2026</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1008,22 +1077,23 @@
           <t>City Sports Complex</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
+      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Group B Winner</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
+          <t>Group A Runner-up</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
           <t>Semi Final 2</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
+      <c r="I15" t="inlineStr">
         <is>
           <t>T20</t>
         </is>
@@ -1035,12 +1105,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>08 Nov 2026</t>
+          <t>23 Oct 2026</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>02:00 PM</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1048,22 +1118,23 @@
           <t>City Sports Complex</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
+      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Winner SF1</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
+          <t>Winner SF2</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
           <t>Final</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="I16" t="inlineStr">
         <is>
           <t>T20</t>
         </is>
@@ -1080,11 +1151,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="120" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="120" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1095,6 +1167,11 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>Players</t>
         </is>
       </c>
@@ -1107,6 +1184,11 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>Aarav A1, Vivaan A2, Aditya A3, Arjun A4, Reyansh A5, Kabir A6, Ishaan A7, Rohan A8, Dhruv A9, Kunal A10, Yash A11</t>
         </is>
       </c>
@@ -1119,6 +1201,11 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
           <t>Atharv B1, Shaurya B2, Vihaan B3, Ayaan B4, Krish B5, Rudra B6, Om B7, Dev B8, Arnav B9, Parth B10, Neel B11</t>
         </is>
       </c>
@@ -1131,6 +1218,11 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
           <t>Tanish C1, Harsh C2, Aarav C3, Vivaan C4, Aditya C5, Arjun C6, Reyansh C7, Kabir C8, Ishaan C9, Rohan C10, Dhruv C11</t>
         </is>
       </c>
@@ -1143,6 +1235,11 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
           <t>Kunal D1, Yash D2, Atharv D3, Shaurya D4, Vihaan D5, Ayaan D6, Krish D7, Rudra D8, Om D9, Dev D10, Arnav D11</t>
         </is>
       </c>
@@ -1155,6 +1252,11 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
           <t>Parth E1, Neel E2, Tanish E3, Harsh E4, Aarav E5, Vivaan E6, Aditya E7, Arjun E8, Reyansh E9, Kabir E10, Ishaan E11</t>
         </is>
       </c>
@@ -1167,6 +1269,11 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
           <t>Rohan F1, Dhruv F2, Kunal F3, Yash F4, Atharv F5, Shaurya F6, Vihaan F7, Ayaan F8, Krish F9, Rudra F10, Om F11</t>
         </is>
       </c>
@@ -1179,6 +1286,11 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
           <t>Dev G1, Arnav G2, Parth G3, Neel G4, Tanish G5, Harsh G6, Aarav G7, Vivaan G8, Aditya G9, Arjun G10, Reyansh G11</t>
         </is>
       </c>
@@ -1191,7 +1303,180 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
           <t>Kabir H1, Ishaan H2, Rohan H3, Dhruv H4, Kunal H5, Yash H6, Atharv H7, Shaurya H8, Vihaan H9, Ayaan H10, Krish H11</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Match No</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Batted First</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Team A Runs</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Team A Wickets</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Team A Overs</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Team B Runs</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Team B Wickets</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Team B Overs</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Winner</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Player of the Match</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Match No</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Team</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Runs</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Balls</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Fours</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Sixes</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Overs Bowled</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Runs Conceded</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Wickets</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Catches</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add results, points table, player stats and a 7-day tournament simulator (#4)
Claude-Session: https://claude.ai/code/session_015MsuMnBjqU5knhALJ8GpAM

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cricket-whatsapp-helpdesk/tournament-fixtures-template.xlsx
+++ b/cricket-whatsapp-helpdesk/tournament-fixtures-template.xlsx
@@ -9,6 +9,8 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fixtures" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Squads" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Results" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Player Stats" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -414,17 +416,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:I16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -450,20 +453,25 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>Team A</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Team B</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Stage</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Format</t>
         </is>
@@ -475,7 +483,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>01 Nov 2026</t>
+          <t>17 Oct 2026</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -490,20 +498,25 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
           <t>Royal Strikers</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>Thunder Kings</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>League</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>T20</t>
         </is>
@@ -515,12 +528,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>01 Nov 2026</t>
+          <t>17 Oct 2026</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>01:30 PM</t>
+          <t>08:00 AM</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -530,7 +543,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Royal Strikers</t>
+          <t>A</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -540,10 +553,15 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
+          <t>Blue Warriors</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
           <t>League</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>T20</t>
         </is>
@@ -555,35 +573,40 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>02 Nov 2026</t>
+          <t>17 Oct 2026</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>01:30 PM</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>City Sports Complex</t>
+          <t>Academy Ground A</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Royal Strikers</t>
+          <t>B</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Blue Warriors</t>
+          <t>Eagle Eleven</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
+          <t>Lion Hearts</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
           <t>League</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>T20</t>
         </is>
@@ -595,12 +618,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>02 Nov 2026</t>
+          <t>18 Oct 2026</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>01:30 PM</t>
+          <t>08:00 AM</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -610,20 +633,25 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Royal Strikers</t>
+          <t>B</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Eagle Eleven</t>
+          <t>Storm Riders</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
+          <t>Golden Titans</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
           <t>League</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>T20</t>
         </is>
@@ -635,7 +663,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>03 Nov 2026</t>
+          <t>18 Oct 2026</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -650,20 +678,25 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
           <t>Royal Strikers</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>Lion Hearts</t>
-        </is>
-      </c>
       <c r="G6" t="inlineStr">
         <is>
+          <t>Super Smashers</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
           <t>League</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>T20</t>
         </is>
@@ -675,7 +708,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>03 Nov 2026</t>
+          <t>18 Oct 2026</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -685,25 +718,30 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>City Sports Complex</t>
+          <t>Academy Ground A</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Royal Strikers</t>
+          <t>A</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Storm Riders</t>
+          <t>Thunder Kings</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
+          <t>Blue Warriors</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
           <t>League</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>T20</t>
         </is>
@@ -715,7 +753,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>04 Nov 2026</t>
+          <t>19 Oct 2026</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -730,20 +768,25 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Royal Strikers</t>
+          <t>B</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Golden Titans</t>
+          <t>Eagle Eleven</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
+          <t>Storm Riders</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
           <t>League</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>T20</t>
         </is>
@@ -755,12 +798,12 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>04 Nov 2026</t>
+          <t>19 Oct 2026</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>01:30 PM</t>
+          <t>08:00 AM</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -770,20 +813,25 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Thunder Kings</t>
+          <t>B</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Super Smashers</t>
+          <t>Lion Hearts</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
+          <t>Golden Titans</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
           <t>League</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>T20</t>
         </is>
@@ -795,35 +843,40 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>05 Nov 2026</t>
+          <t>19 Oct 2026</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>01:30 PM</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>City Sports Complex</t>
+          <t>Academy Ground A</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Thunder Kings</t>
+          <t>A</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
+          <t>Royal Strikers</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
           <t>Blue Warriors</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>League</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="I10" t="inlineStr">
         <is>
           <t>T20</t>
         </is>
@@ -835,12 +888,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>05 Nov 2026</t>
+          <t>20 Oct 2026</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>01:30 PM</t>
+          <t>08:00 AM</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -850,20 +903,25 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
           <t>Thunder Kings</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>Eagle Eleven</t>
-        </is>
-      </c>
       <c r="G11" t="inlineStr">
         <is>
+          <t>Super Smashers</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
           <t>League</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="I11" t="inlineStr">
         <is>
           <t>T20</t>
         </is>
@@ -875,7 +933,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>06 Nov 2026</t>
+          <t>20 Oct 2026</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -890,20 +948,25 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Thunder Kings</t>
+          <t>B</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Lion Hearts</t>
+          <t>Eagle Eleven</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
+          <t>Golden Titans</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
           <t>League</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>T20</t>
         </is>
@@ -915,7 +978,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>06 Nov 2026</t>
+          <t>20 Oct 2026</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -925,25 +988,30 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>City Sports Complex</t>
+          <t>Academy Ground A</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Thunder Kings</t>
+          <t>B</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
+          <t>Lion Hearts</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
           <t>Storm Riders</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="H13" t="inlineStr">
         <is>
           <t>League</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="I13" t="inlineStr">
         <is>
           <t>T20</t>
         </is>
@@ -955,7 +1023,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>07 Nov 2026</t>
+          <t>22 Oct 2026</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -968,22 +1036,23 @@
           <t>City Sports Complex</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
+      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Group A Winner</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
+          <t>Group B Runner-up</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
           <t>Semi Final 1</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
+      <c r="I14" t="inlineStr">
         <is>
           <t>T20</t>
         </is>
@@ -995,7 +1064,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>07 Nov 2026</t>
+          <t>22 Oct 2026</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1008,22 +1077,23 @@
           <t>City Sports Complex</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
+      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Group B Winner</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
+          <t>Group A Runner-up</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
           <t>Semi Final 2</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
+      <c r="I15" t="inlineStr">
         <is>
           <t>T20</t>
         </is>
@@ -1035,12 +1105,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>08 Nov 2026</t>
+          <t>23 Oct 2026</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>08:00 AM</t>
+          <t>02:00 PM</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1048,22 +1118,23 @@
           <t>City Sports Complex</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>TBD</t>
-        </is>
-      </c>
+      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Winner SF1</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
+          <t>Winner SF2</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
           <t>Final</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
+      <c r="I16" t="inlineStr">
         <is>
           <t>T20</t>
         </is>
@@ -1080,11 +1151,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="120" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="120" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1095,6 +1167,11 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>Group</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
           <t>Players</t>
         </is>
       </c>
@@ -1107,6 +1184,11 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
           <t>Aarav A1, Vivaan A2, Aditya A3, Arjun A4, Reyansh A5, Kabir A6, Ishaan A7, Rohan A8, Dhruv A9, Kunal A10, Yash A11</t>
         </is>
       </c>
@@ -1119,6 +1201,11 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
           <t>Atharv B1, Shaurya B2, Vihaan B3, Ayaan B4, Krish B5, Rudra B6, Om B7, Dev B8, Arnav B9, Parth B10, Neel B11</t>
         </is>
       </c>
@@ -1131,6 +1218,11 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
           <t>Tanish C1, Harsh C2, Aarav C3, Vivaan C4, Aditya C5, Arjun C6, Reyansh C7, Kabir C8, Ishaan C9, Rohan C10, Dhruv C11</t>
         </is>
       </c>
@@ -1143,6 +1235,11 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
           <t>Kunal D1, Yash D2, Atharv D3, Shaurya D4, Vihaan D5, Ayaan D6, Krish D7, Rudra D8, Om D9, Dev D10, Arnav D11</t>
         </is>
       </c>
@@ -1155,6 +1252,11 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
           <t>Parth E1, Neel E2, Tanish E3, Harsh E4, Aarav E5, Vivaan E6, Aditya E7, Arjun E8, Reyansh E9, Kabir E10, Ishaan E11</t>
         </is>
       </c>
@@ -1167,6 +1269,11 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
           <t>Rohan F1, Dhruv F2, Kunal F3, Yash F4, Atharv F5, Shaurya F6, Vihaan F7, Ayaan F8, Krish F9, Rudra F10, Om F11</t>
         </is>
       </c>
@@ -1179,6 +1286,11 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
           <t>Dev G1, Arnav G2, Parth G3, Neel G4, Tanish G5, Harsh G6, Aarav G7, Vivaan G8, Aditya G9, Arjun G10, Reyansh G11</t>
         </is>
       </c>
@@ -1191,7 +1303,180 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
           <t>Kabir H1, Ishaan H2, Rohan H3, Dhruv H4, Kunal H5, Yash H6, Atharv H7, Shaurya H8, Vihaan H9, Ayaan H10, Krish H11</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Match No</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Batted First</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Team A Runs</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Team A Wickets</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Team A Overs</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Team B Runs</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Team B Wickets</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Team B Overs</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Winner</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Player of the Match</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Match No</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Team</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Runs</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Balls</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Fours</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Sixes</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Overs Bowled</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Runs Conceded</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Wickets</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Catches</t>
         </is>
       </c>
     </row>

</xml_diff>